<commit_message>
feat(data): 支持导出 protobuf 二进制数据
</commit_message>
<xml_diff>
--- a/assets/xls/升级.xlsx
+++ b/assets/xls/升级.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="21315" windowHeight="10680" tabRatio="535"/>
+    <workbookView windowWidth="21555" windowHeight="11265" tabRatio="535"/>
   </bookViews>
   <sheets>
     <sheet name="Upgrade" sheetId="7" r:id="rId1"/>
@@ -50,17 +50,40 @@
         </r>
       </text>
     </comment>
+    <comment ref="C1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="宋体"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">
+fk:Resource.ID=Item.ID;
+</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="28">
   <si>
     <t>ID</t>
   </si>
   <si>
-    <t>Cost</t>
+    <t>Costs</t>
+  </si>
+  <si>
+    <t>Rewards</t>
+  </si>
+  <si>
+    <t>Attribs</t>
+  </si>
+  <si>
+    <t>Icons</t>
   </si>
   <si>
     <t>unique int32</t>
@@ -69,6 +92,12 @@
     <t>repeated Resource</t>
   </si>
   <si>
+    <t>repeated int32</t>
+  </si>
+  <si>
+    <t>repeated string</t>
+  </si>
+  <si>
     <t>cs</t>
   </si>
   <si>
@@ -78,10 +107,52 @@
     <t>消耗材料</t>
   </si>
   <si>
-    <t>8|5,10|10</t>
-  </si>
-  <si>
-    <t>9|15,10|20</t>
+    <t>奖励材料</t>
+  </si>
+  <si>
+    <t>属性列表</t>
+  </si>
+  <si>
+    <t>图标列表</t>
+  </si>
+  <si>
+    <t>8|5;10|10</t>
+  </si>
+  <si>
+    <t>5;8;10</t>
+  </si>
+  <si>
+    <t>aa;bb;cc</t>
+  </si>
+  <si>
+    <t>9|15;10|20</t>
+  </si>
+  <si>
+    <t>5;8;11</t>
+  </si>
+  <si>
+    <t>5;8;12</t>
+  </si>
+  <si>
+    <t>5;8;13</t>
+  </si>
+  <si>
+    <t>5;8;14</t>
+  </si>
+  <si>
+    <t>5;8;15</t>
+  </si>
+  <si>
+    <t>5;8;16</t>
+  </si>
+  <si>
+    <t>5;8;17</t>
+  </si>
+  <si>
+    <t>5;8;18</t>
+  </si>
+  <si>
+    <t>5;8;19</t>
   </si>
 </sst>
 </file>
@@ -1076,124 +1147,252 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B14"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="1"/>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="15.375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="21.625" style="2" customWidth="1"/>
-    <col min="3" max="16384" width="9" style="2"/>
+    <col min="2" max="3" width="21.625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="17.875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="19.125" style="2" customWidth="1"/>
+    <col min="6" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:2">
+    <row r="1" s="1" customFormat="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="2" s="1" customFormat="1" spans="1:2">
+    <row r="2" s="1" customFormat="1" spans="1:5">
       <c r="A2" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>3</v>
+        <v>6</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="3" s="1" customFormat="1" spans="1:2">
+    <row r="3" s="1" customFormat="1" spans="1:5">
       <c r="A3" s="1" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>4</v>
+        <v>9</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
-    <row r="4" s="1" customFormat="1" spans="1:2">
+    <row r="4" s="1" customFormat="1" spans="1:5">
       <c r="A4" s="1" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>6</v>
+        <v>11</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
-    <row r="5" s="1" customFormat="1" spans="1:2">
+    <row r="5" s="1" customFormat="1" spans="1:5">
       <c r="A5" s="2">
         <v>1</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>7</v>
+        <v>15</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:5">
       <c r="A6" s="2">
         <v>2</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>8</v>
+        <v>18</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:5">
       <c r="A7" s="2">
         <v>3</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>7</v>
+        <v>15</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:5">
       <c r="A8" s="2">
         <v>4</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>8</v>
+        <v>18</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:5">
       <c r="A9" s="2">
         <v>5</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>7</v>
+        <v>15</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:5">
       <c r="A10" s="2">
         <v>6</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>8</v>
+        <v>18</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:5">
       <c r="A11" s="2">
         <v>7</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>7</v>
+        <v>15</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:5">
       <c r="A12" s="2">
         <v>8</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>8</v>
+        <v>18</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:5">
       <c r="A13" s="2">
         <v>9</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>7</v>
+        <v>15</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:5">
       <c r="A14" s="2">
         <v>10</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>8</v>
+        <v>18</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(codegen): 完善 protobuf 类型代码生成
</commit_message>
<xml_diff>
--- a/assets/xls/升级.xlsx
+++ b/assets/xls/升级.xlsx
@@ -69,12 +69,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="30">
   <si>
     <t>ID</t>
   </si>
   <si>
-    <t>Costs</t>
+    <t>Cost</t>
   </si>
   <si>
     <t>Rewards</t>
@@ -89,6 +89,9 @@
     <t>unique int32</t>
   </si>
   <si>
+    <t>Resource</t>
+  </si>
+  <si>
     <t>repeated Resource</t>
   </si>
   <si>
@@ -116,19 +119,22 @@
     <t>图标列表</t>
   </si>
   <si>
+    <t>9|15</t>
+  </si>
+  <si>
+    <t>9|15;10|20</t>
+  </si>
+  <si>
+    <t>5;8;11</t>
+  </si>
+  <si>
+    <t>aa;bb;cc</t>
+  </si>
+  <si>
+    <t>8|5</t>
+  </si>
+  <si>
     <t>8|5;10|10</t>
-  </si>
-  <si>
-    <t>5;8;10</t>
-  </si>
-  <si>
-    <t>aa;bb;cc</t>
-  </si>
-  <si>
-    <t>9|15;10|20</t>
-  </si>
-  <si>
-    <t>5;8;11</t>
   </si>
   <si>
     <t>5;8;12</t>
@@ -1151,7 +1157,8 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="15.375" style="2" customWidth="1"/>
-    <col min="2" max="3" width="21.625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="10.375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="21.625" style="2" customWidth="1"/>
     <col min="4" max="4" width="17.875" style="2" customWidth="1"/>
     <col min="5" max="5" width="19.125" style="2" customWidth="1"/>
     <col min="6" max="16384" width="9" style="2"/>
@@ -1182,81 +1189,73 @@
         <v>6</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" s="1" customFormat="1" spans="1:5">
       <c r="A3" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" s="1" customFormat="1" spans="1:5">
       <c r="A4" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" s="1" customFormat="1" spans="1:5">
       <c r="A5" s="2">
         <v>1</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>17</v>
-      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="2">
         <v>2</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>19</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -1264,16 +1263,16 @@
         <v>3</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -1281,16 +1280,16 @@
         <v>4</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -1298,16 +1297,16 @@
         <v>5</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -1315,16 +1314,16 @@
         <v>6</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -1332,16 +1331,16 @@
         <v>7</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -1349,16 +1348,16 @@
         <v>8</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -1366,16 +1365,16 @@
         <v>9</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -1383,16 +1382,16 @@
         <v>10</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(parser): 支持 float 和 double 字段
</commit_message>
<xml_diff>
--- a/assets/xls/升级.xlsx
+++ b/assets/xls/升级.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="21555" windowHeight="11265" tabRatio="535"/>
+    <workbookView windowWidth="16380" windowHeight="8235" tabRatio="535"/>
   </bookViews>
   <sheets>
     <sheet name="Upgrade" sheetId="7" r:id="rId1"/>
@@ -86,7 +86,7 @@
     <t>Icons</t>
   </si>
   <si>
-    <t>unique int32</t>
+    <t>pk int32</t>
   </si>
   <si>
     <t>Resource</t>

</xml_diff>